<commit_message>
Adding the sales report with images & pdf file
</commit_message>
<xml_diff>
--- a/Excel/Book2.xlsx
+++ b/Excel/Book2.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\j-l-data-science-data-analytics\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{979C11CE-BAD5-4ED2-9D5B-001E049A1C27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7595D284-73C5-4278-9572-DDF04F7D8383}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="42">
   <si>
     <t>Grade Book</t>
   </si>
@@ -122,12 +123,51 @@
   <si>
     <t>AVERAGE</t>
   </si>
+  <si>
+    <t>Career Decision Time</t>
+  </si>
+  <si>
+    <t>Job</t>
+  </si>
+  <si>
+    <t>Jafar-Loka-01</t>
+  </si>
+  <si>
+    <t>Jafar-Loka-02</t>
+  </si>
+  <si>
+    <t>Jafar-Loka-03</t>
+  </si>
+  <si>
+    <t>Jafar-Loka-04</t>
+  </si>
+  <si>
+    <t>Jafar-Loka-05</t>
+  </si>
+  <si>
+    <t>Pay</t>
+  </si>
+  <si>
+    <t>Job Market</t>
+  </si>
+  <si>
+    <t>Enjoyment</t>
+  </si>
+  <si>
+    <t>My Talent</t>
+  </si>
+  <si>
+    <t>Schooling</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -142,13 +182,74 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="11"/>
+      <color theme="9" tint="-0.249977111117893"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFABF84"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -164,39 +265,32 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment textRotation="45"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="9">
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="4">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -237,38 +331,13 @@
         </patternFill>
       </fill>
     </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFFABF84"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -507,52 +576,52 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="17"/>
                 <c:pt idx="0">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>6</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>5</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>10</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>10</c:v>
                 </c:pt>
                 <c:pt idx="4">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="6">
                   <c:v>7</c:v>
                 </c:pt>
-                <c:pt idx="5">
-                  <c:v>8</c:v>
-                </c:pt>
-                <c:pt idx="6">
+                <c:pt idx="7">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="8">
                   <c:v>9</c:v>
                 </c:pt>
-                <c:pt idx="7">
-                  <c:v>9</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>10</c:v>
-                </c:pt>
                 <c:pt idx="9">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="10">
                   <c:v>5</c:v>
                 </c:pt>
-                <c:pt idx="10">
-                  <c:v>7</c:v>
-                </c:pt>
                 <c:pt idx="11">
-                  <c:v>9</c:v>
+                  <c:v>6</c:v>
                 </c:pt>
                 <c:pt idx="12">
                   <c:v>10</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>5</c:v>
+                  <c:v>9</c:v>
                 </c:pt>
                 <c:pt idx="14">
                   <c:v>8</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>7</c:v>
+                  <c:v>6</c:v>
                 </c:pt>
                 <c:pt idx="16">
                   <c:v>7</c:v>
@@ -902,55 +971,55 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="17"/>
                 <c:pt idx="0">
-                  <c:v>11</c:v>
+                  <c:v>20</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>14</c:v>
+                  <c:v>20</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>17</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>15</c:v>
+                  <c:v>14</c:v>
                 </c:pt>
                 <c:pt idx="4">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>13</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>13</c:v>
+                </c:pt>
+                <c:pt idx="10">
                   <c:v>11</c:v>
                 </c:pt>
-                <c:pt idx="5">
-                  <c:v>10</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>10</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>11</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>16</c:v>
-                </c:pt>
-                <c:pt idx="9">
+                <c:pt idx="11">
                   <c:v>19</c:v>
                 </c:pt>
-                <c:pt idx="10">
-                  <c:v>20</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>17</c:v>
-                </c:pt>
                 <c:pt idx="12">
-                  <c:v>20</c:v>
+                  <c:v>18</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>10</c:v>
+                  <c:v>14</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>15</c:v>
+                  <c:v>12</c:v>
                 </c:pt>
                 <c:pt idx="15">
                   <c:v>16</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>15</c:v>
+                  <c:v>19</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1320,55 +1389,55 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="17"/>
                 <c:pt idx="0">
-                  <c:v>75</c:v>
+                  <c:v>80</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>96</c:v>
+                  <c:v>74</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>69</c:v>
+                  <c:v>54</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>95</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>57</c:v>
+                  <c:v>93</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>70</c:v>
+                  <c:v>53</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>92</c:v>
+                  <c:v>59</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>50</c:v>
+                  <c:v>56</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>92</c:v>
+                  <c:v>80</c:v>
                 </c:pt>
                 <c:pt idx="9">
                   <c:v>60</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>96</c:v>
+                  <c:v>69</c:v>
                 </c:pt>
                 <c:pt idx="11">
+                  <c:v>97</c:v>
+                </c:pt>
+                <c:pt idx="12">
                   <c:v>95</c:v>
                 </c:pt>
-                <c:pt idx="12">
-                  <c:v>82</c:v>
-                </c:pt>
                 <c:pt idx="13">
-                  <c:v>77</c:v>
+                  <c:v>83</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>96</c:v>
+                  <c:v>84</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>57</c:v>
+                  <c:v>64</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>69</c:v>
+                  <c:v>89</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3718,6 +3787,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:M24"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3802,39 +3874,39 @@
       </c>
       <c r="C4">
         <f ca="1">RANDBETWEEN(5, 10)</f>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D4">
         <f ca="1">RANDBETWEEN(10, 20)</f>
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="E4">
         <f ca="1">RANDBETWEEN(50, 100)</f>
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="F4">
         <f ca="1">RANDBETWEEN(0, 1)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H4" s="1">
         <f ca="1">C4/C$2</f>
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="I4" s="1">
         <f ca="1">D4/D$2</f>
-        <v>0.55000000000000004</v>
+        <v>1</v>
       </c>
       <c r="J4" s="1">
         <f t="shared" ref="J4:K19" ca="1" si="0">E4/E$2</f>
-        <v>0.75</v>
+        <v>0.8</v>
       </c>
       <c r="K4" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M4" s="1" t="b">
         <f ca="1">OR(H4&lt;0.5, I4&lt;0.5, J4&lt;0.5, K4&lt;0.5)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
@@ -3846,15 +3918,15 @@
       </c>
       <c r="C5">
         <f t="shared" ref="C5:C20" ca="1" si="1">RANDBETWEEN(5, 10)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D5">
         <f t="shared" ref="D5:D20" ca="1" si="2">RANDBETWEEN(10, 20)</f>
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="E5">
         <f t="shared" ref="E5:E20" ca="1" si="3">RANDBETWEEN(50, 100)</f>
-        <v>96</v>
+        <v>74</v>
       </c>
       <c r="F5">
         <f t="shared" ref="F5:F20" ca="1" si="4">RANDBETWEEN(0, 1)</f>
@@ -3862,15 +3934,15 @@
       </c>
       <c r="H5" s="1">
         <f t="shared" ref="H5:I20" ca="1" si="5">C5/C$2</f>
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="I5" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>0.7</v>
+        <v>1</v>
       </c>
       <c r="J5" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>0.96</v>
+        <v>0.74</v>
       </c>
       <c r="K5" s="1">
         <f t="shared" ca="1" si="0"/>
@@ -3890,7 +3962,7 @@
       </c>
       <c r="C6">
         <f t="shared" ca="1" si="1"/>
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D6">
         <f t="shared" ca="1" si="2"/>
@@ -3898,7 +3970,7 @@
       </c>
       <c r="E6">
         <f t="shared" ca="1" si="3"/>
-        <v>69</v>
+        <v>54</v>
       </c>
       <c r="F6">
         <f t="shared" ca="1" si="4"/>
@@ -3906,7 +3978,7 @@
       </c>
       <c r="H6" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="I6" s="1">
         <f t="shared" ca="1" si="5"/>
@@ -3914,7 +3986,7 @@
       </c>
       <c r="J6" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>0.69</v>
+        <v>0.54</v>
       </c>
       <c r="K6" s="1">
         <f t="shared" ca="1" si="0"/>
@@ -3938,7 +4010,7 @@
       </c>
       <c r="D7">
         <f t="shared" ca="1" si="2"/>
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E7">
         <f t="shared" ca="1" si="3"/>
@@ -3954,7 +4026,7 @@
       </c>
       <c r="I7" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>0.75</v>
+        <v>0.7</v>
       </c>
       <c r="J7" s="1">
         <f t="shared" ca="1" si="0"/>
@@ -3978,39 +4050,39 @@
       </c>
       <c r="C8">
         <f t="shared" ca="1" si="1"/>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D8">
         <f t="shared" ca="1" si="2"/>
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="E8">
         <f t="shared" ca="1" si="3"/>
-        <v>57</v>
+        <v>93</v>
       </c>
       <c r="F8">
         <f t="shared" ca="1" si="4"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H8" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
       <c r="I8" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>0.55000000000000004</v>
+        <v>0.9</v>
       </c>
       <c r="J8" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>0.56999999999999995</v>
+        <v>0.93</v>
       </c>
       <c r="K8" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M8" s="1" t="b">
         <f t="shared" ca="1" si="6"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
@@ -4022,39 +4094,39 @@
       </c>
       <c r="C9">
         <f t="shared" ca="1" si="1"/>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D9">
         <f t="shared" ca="1" si="2"/>
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E9">
         <f t="shared" ca="1" si="3"/>
-        <v>70</v>
+        <v>53</v>
       </c>
       <c r="F9">
         <f t="shared" ca="1" si="4"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H9" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="I9" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>0.5</v>
+        <v>0.8</v>
       </c>
       <c r="J9" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>0.7</v>
+        <v>0.53</v>
       </c>
       <c r="K9" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M9" s="1" t="b">
         <f t="shared" ca="1" si="6"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
@@ -4066,15 +4138,15 @@
       </c>
       <c r="C10">
         <f t="shared" ca="1" si="1"/>
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D10">
         <f t="shared" ca="1" si="2"/>
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="E10">
         <f t="shared" ca="1" si="3"/>
-        <v>92</v>
+        <v>59</v>
       </c>
       <c r="F10">
         <f t="shared" ca="1" si="4"/>
@@ -4082,15 +4154,15 @@
       </c>
       <c r="H10" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>0.9</v>
+        <v>0.7</v>
       </c>
       <c r="I10" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>0.5</v>
+        <v>0.9</v>
       </c>
       <c r="J10" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>0.92</v>
+        <v>0.59</v>
       </c>
       <c r="K10" s="1">
         <f t="shared" ca="1" si="0"/>
@@ -4110,39 +4182,39 @@
       </c>
       <c r="C11">
         <f t="shared" ca="1" si="1"/>
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="D11">
         <f t="shared" ca="1" si="2"/>
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E11">
         <f t="shared" ca="1" si="3"/>
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="F11">
         <f t="shared" ca="1" si="4"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H11" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>0.9</v>
+        <v>0.5</v>
       </c>
       <c r="I11" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>0.55000000000000004</v>
+        <v>0.65</v>
       </c>
       <c r="J11" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>0.5</v>
+        <v>0.56000000000000005</v>
       </c>
       <c r="K11" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M11" s="1" t="b">
         <f t="shared" ca="1" si="6"/>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
@@ -4154,15 +4226,15 @@
       </c>
       <c r="C12">
         <f t="shared" ca="1" si="1"/>
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D12">
         <f t="shared" ca="1" si="2"/>
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="E12">
         <f t="shared" ca="1" si="3"/>
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="F12">
         <f t="shared" ca="1" si="4"/>
@@ -4170,15 +4242,15 @@
       </c>
       <c r="H12" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="I12" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
       <c r="J12" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>0.92</v>
+        <v>0.8</v>
       </c>
       <c r="K12" s="1">
         <f t="shared" ca="1" si="0"/>
@@ -4198,11 +4270,11 @@
       </c>
       <c r="C13">
         <f t="shared" ca="1" si="1"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D13">
         <f t="shared" ca="1" si="2"/>
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="E13">
         <f t="shared" ca="1" si="3"/>
@@ -4214,11 +4286,11 @@
       </c>
       <c r="H13" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="I13" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>0.95</v>
+        <v>0.65</v>
       </c>
       <c r="J13" s="1">
         <f t="shared" ca="1" si="0"/>
@@ -4242,39 +4314,39 @@
       </c>
       <c r="C14">
         <f t="shared" ca="1" si="1"/>
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D14">
         <f t="shared" ca="1" si="2"/>
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="E14">
         <f t="shared" ca="1" si="3"/>
-        <v>96</v>
+        <v>69</v>
       </c>
       <c r="F14">
         <f t="shared" ca="1" si="4"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H14" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="I14" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>1</v>
+        <v>0.55000000000000004</v>
       </c>
       <c r="J14" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>0.96</v>
+        <v>0.69</v>
       </c>
       <c r="K14" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M14" s="1" t="b">
         <f t="shared" ca="1" si="6"/>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
@@ -4286,39 +4358,39 @@
       </c>
       <c r="C15">
         <f t="shared" ca="1" si="1"/>
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D15">
         <f t="shared" ca="1" si="2"/>
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="E15">
         <f t="shared" ca="1" si="3"/>
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="F15">
         <f t="shared" ca="1" si="4"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H15" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>0.9</v>
+        <v>0.6</v>
       </c>
       <c r="I15" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>0.85</v>
+        <v>0.95</v>
       </c>
       <c r="J15" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>0.95</v>
+        <v>0.97</v>
       </c>
       <c r="K15" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M15" s="1" t="b">
         <f t="shared" ca="1" si="6"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.25">
@@ -4334,11 +4406,11 @@
       </c>
       <c r="D16">
         <f t="shared" ca="1" si="2"/>
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E16">
         <f t="shared" ca="1" si="3"/>
-        <v>82</v>
+        <v>95</v>
       </c>
       <c r="F16">
         <f t="shared" ca="1" si="4"/>
@@ -4350,11 +4422,11 @@
       </c>
       <c r="I16" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="J16" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>0.82</v>
+        <v>0.95</v>
       </c>
       <c r="K16" s="1">
         <f t="shared" ca="1" si="0"/>
@@ -4374,39 +4446,39 @@
       </c>
       <c r="C17">
         <f t="shared" ca="1" si="1"/>
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="D17">
         <f t="shared" ca="1" si="2"/>
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="E17">
         <f t="shared" ca="1" si="3"/>
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="F17">
         <f t="shared" ca="1" si="4"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H17" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>0.5</v>
+        <v>0.9</v>
       </c>
       <c r="I17" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="J17" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>0.77</v>
+        <v>0.83</v>
       </c>
       <c r="K17" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M17" s="1" t="b">
         <f t="shared" ca="1" si="6"/>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.25">
@@ -4422,15 +4494,15 @@
       </c>
       <c r="D18">
         <f t="shared" ca="1" si="2"/>
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="E18">
         <f t="shared" ca="1" si="3"/>
-        <v>96</v>
+        <v>84</v>
       </c>
       <c r="F18">
         <f t="shared" ca="1" si="4"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H18" s="1">
         <f t="shared" ca="1" si="5"/>
@@ -4438,19 +4510,19 @@
       </c>
       <c r="I18" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>0.75</v>
+        <v>0.6</v>
       </c>
       <c r="J18" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>0.96</v>
+        <v>0.84</v>
       </c>
       <c r="K18" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M18" s="1" t="b">
         <f t="shared" ca="1" si="6"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.25">
@@ -4462,7 +4534,7 @@
       </c>
       <c r="C19">
         <f t="shared" ca="1" si="1"/>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D19">
         <f t="shared" ca="1" si="2"/>
@@ -4470,15 +4542,15 @@
       </c>
       <c r="E19">
         <f t="shared" ca="1" si="3"/>
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="F19">
         <f t="shared" ca="1" si="4"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H19" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
       <c r="I19" s="1">
         <f t="shared" ca="1" si="5"/>
@@ -4486,15 +4558,15 @@
       </c>
       <c r="J19" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>0.56999999999999995</v>
+        <v>0.64</v>
       </c>
       <c r="K19" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M19" s="1" t="b">
         <f t="shared" ca="1" si="6"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.25">
@@ -4510,11 +4582,11 @@
       </c>
       <c r="D20">
         <f t="shared" ca="1" si="2"/>
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E20">
         <f t="shared" ca="1" si="3"/>
-        <v>69</v>
+        <v>89</v>
       </c>
       <c r="F20">
         <f t="shared" ca="1" si="4"/>
@@ -4526,11 +4598,11 @@
       </c>
       <c r="I20" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>0.75</v>
+        <v>0.95</v>
       </c>
       <c r="J20" s="1">
         <f t="shared" ref="J20" ca="1" si="7">E20/E$2</f>
-        <v>0.69</v>
+        <v>0.89</v>
       </c>
       <c r="K20" s="1">
         <f t="shared" ref="K20" ca="1" si="8">F20/F$2</f>
@@ -4550,12 +4622,12 @@
         <v>10</v>
       </c>
       <c r="D22">
-        <f t="shared" ref="D22:F22" ca="1" si="9">MAX(D4:D20)</f>
+        <f t="shared" ref="D22:E22" ca="1" si="9">MAX(D4:D20)</f>
         <v>20</v>
       </c>
       <c r="E22">
         <f t="shared" ca="1" si="9"/>
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="F22">
         <f t="shared" ref="F22" ca="1" si="10">MAX(F4:F20)</f>
@@ -4571,7 +4643,7 @@
       </c>
       <c r="J22" s="1">
         <f t="shared" ca="1" si="11"/>
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="K22" s="1">
         <f t="shared" ca="1" si="11"/>
@@ -4587,12 +4659,12 @@
         <v>5</v>
       </c>
       <c r="D23">
-        <f t="shared" ref="D23:F23" ca="1" si="12">MIN(D4:D20)</f>
-        <v>10</v>
+        <f t="shared" ref="D23:E23" ca="1" si="12">MIN(D4:D20)</f>
+        <v>11</v>
       </c>
       <c r="E23">
         <f t="shared" ca="1" si="12"/>
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="F23">
         <f t="shared" ref="F23" ca="1" si="13">MIN(F4:F20)</f>
@@ -4604,11 +4676,11 @@
       </c>
       <c r="I23" s="1">
         <f t="shared" ref="I23:K23" ca="1" si="14">MIN(I4:I20)</f>
-        <v>0.5</v>
+        <v>0.55000000000000004</v>
       </c>
       <c r="J23" s="1">
         <f t="shared" ca="1" si="14"/>
-        <v>0.5</v>
+        <v>0.53</v>
       </c>
       <c r="K23" s="1">
         <f t="shared" ca="1" si="14"/>
@@ -4621,35 +4693,35 @@
       </c>
       <c r="C24" s="3">
         <f ca="1">AVERAGE(C4:C21)</f>
-        <v>7.7647058823529411</v>
+        <v>7</v>
       </c>
       <c r="D24" s="3">
-        <f t="shared" ref="D24:F24" ca="1" si="15">AVERAGE(D4:D21)</f>
-        <v>14.529411764705882</v>
+        <f t="shared" ref="D24:E24" ca="1" si="15">AVERAGE(D4:D21)</f>
+        <v>16</v>
       </c>
       <c r="E24" s="3">
         <f t="shared" ca="1" si="15"/>
-        <v>78.117647058823536</v>
+        <v>75.588235294117652</v>
       </c>
       <c r="F24" s="3">
         <f t="shared" ref="F24" ca="1" si="16">AVERAGE(F4:F21)</f>
-        <v>0.58823529411764708</v>
+        <v>0.41176470588235292</v>
       </c>
       <c r="H24" s="1">
         <f ca="1">AVERAGE(H4:H21)</f>
-        <v>0.77647058823529402</v>
+        <v>0.70000000000000007</v>
       </c>
       <c r="I24" s="1">
         <f t="shared" ref="I24:K24" ca="1" si="17">AVERAGE(I4:I21)</f>
-        <v>0.7264705882352942</v>
+        <v>0.79999999999999993</v>
       </c>
       <c r="J24" s="1">
         <f t="shared" ca="1" si="17"/>
-        <v>0.78117647058823525</v>
+        <v>0.75588235294117656</v>
       </c>
       <c r="K24" s="1">
         <f t="shared" ca="1" si="17"/>
-        <v>0.58823529411764708</v>
+        <v>0.41176470588235292</v>
       </c>
     </row>
   </sheetData>
@@ -4693,20 +4765,332 @@
       </iconSet>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H4:K20 M4:M20">
-    <cfRule type="cellIs" dxfId="7" priority="3" operator="lessThan">
+  <conditionalFormatting sqref="M4:M20 H4:K20">
+    <cfRule type="cellIs" dxfId="3" priority="3" operator="lessThan">
       <formula>0.5</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M4:M20">
-    <cfRule type="cellIs" dxfId="3" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
+      <formula>FALSE</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
       <formula>TRUE</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="1" operator="equal">
-      <formula>FALSE</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup paperSize="9" scale="50" orientation="landscape" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D419627-A140-48E5-ACCB-2DB7323EEF90}">
+  <dimension ref="B1:M12"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="22.28515625" customWidth="1"/>
+    <col min="3" max="3" width="13.140625" customWidth="1"/>
+    <col min="4" max="4" width="14.140625" customWidth="1"/>
+    <col min="5" max="5" width="17.85546875" customWidth="1"/>
+    <col min="7" max="7" width="23.85546875" customWidth="1"/>
+    <col min="9" max="9" width="20" customWidth="1"/>
+    <col min="11" max="11" width="20.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="7" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B7" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="C7" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="D7" s="11">
+        <v>3</v>
+      </c>
+      <c r="E7" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="F7" s="12">
+        <v>5</v>
+      </c>
+      <c r="G7" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="H7" s="13">
+        <v>4</v>
+      </c>
+      <c r="I7" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="J7" s="14">
+        <v>3</v>
+      </c>
+      <c r="K7" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="L7" s="15">
+        <v>1</v>
+      </c>
+      <c r="M7" s="10" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="8" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B8" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="C8" s="4">
+        <f ca="1">RANDBETWEEN(1, 5)</f>
+        <v>2</v>
+      </c>
+      <c r="D8" s="4">
+        <f ca="1">D$7*C8</f>
+        <v>6</v>
+      </c>
+      <c r="E8" s="5">
+        <f ca="1">RANDBETWEEN(1, 5)</f>
+        <v>1</v>
+      </c>
+      <c r="F8" s="5">
+        <f ca="1">F$7*E8</f>
+        <v>5</v>
+      </c>
+      <c r="G8" s="6">
+        <f ca="1">RANDBETWEEN(1, 5)</f>
+        <v>5</v>
+      </c>
+      <c r="H8" s="6">
+        <f ca="1">H$7*G8</f>
+        <v>20</v>
+      </c>
+      <c r="I8" s="7">
+        <f ca="1">RANDBETWEEN(1, 5)</f>
+        <v>3</v>
+      </c>
+      <c r="J8" s="7">
+        <f ca="1">J$7*I8</f>
+        <v>9</v>
+      </c>
+      <c r="K8" s="8">
+        <f ca="1">RANDBETWEEN(1, 5)</f>
+        <v>2</v>
+      </c>
+      <c r="L8" s="8">
+        <f ca="1">L$7*K8</f>
+        <v>2</v>
+      </c>
+      <c r="M8" s="9">
+        <f ca="1">SUM(F8,D8,H8,J8,L8)</f>
+        <v>42</v>
+      </c>
+    </row>
+    <row r="9" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B9" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="C9" s="4">
+        <f t="shared" ref="C9:C12" ca="1" si="0">RANDBETWEEN(1, 5)</f>
+        <v>4</v>
+      </c>
+      <c r="D9" s="4">
+        <f t="shared" ref="D9:D12" ca="1" si="1">D$7*C9</f>
+        <v>12</v>
+      </c>
+      <c r="E9" s="5">
+        <f t="shared" ref="E9:E12" ca="1" si="2">RANDBETWEEN(1, 5)</f>
+        <v>1</v>
+      </c>
+      <c r="F9" s="5">
+        <f t="shared" ref="F9:F12" ca="1" si="3">F$7*E9</f>
+        <v>5</v>
+      </c>
+      <c r="G9" s="6">
+        <f t="shared" ref="G9:G12" ca="1" si="4">RANDBETWEEN(1, 5)</f>
+        <v>3</v>
+      </c>
+      <c r="H9" s="6">
+        <f t="shared" ref="H9:H12" ca="1" si="5">H$7*G9</f>
+        <v>12</v>
+      </c>
+      <c r="I9" s="7">
+        <f t="shared" ref="I9:I12" ca="1" si="6">RANDBETWEEN(1, 5)</f>
+        <v>1</v>
+      </c>
+      <c r="J9" s="7">
+        <f t="shared" ref="J9:J12" ca="1" si="7">J$7*I9</f>
+        <v>3</v>
+      </c>
+      <c r="K9" s="8">
+        <f t="shared" ref="K9:L12" ca="1" si="8">RANDBETWEEN(1, 5)</f>
+        <v>4</v>
+      </c>
+      <c r="L9" s="8">
+        <f t="shared" ref="L9:L12" ca="1" si="9">L$7*K9</f>
+        <v>4</v>
+      </c>
+      <c r="M9" s="9">
+        <f ca="1">SUM(F9,D9,H9,J9,L9)</f>
+        <v>36</v>
+      </c>
+    </row>
+    <row r="10" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B10" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="C10" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="D10" s="4">
+        <f t="shared" ca="1" si="1"/>
+        <v>9</v>
+      </c>
+      <c r="E10" s="5">
+        <f t="shared" ca="1" si="2"/>
+        <v>5</v>
+      </c>
+      <c r="F10" s="5">
+        <f t="shared" ca="1" si="3"/>
+        <v>25</v>
+      </c>
+      <c r="G10" s="6">
+        <f t="shared" ca="1" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="H10" s="6">
+        <f t="shared" ca="1" si="5"/>
+        <v>4</v>
+      </c>
+      <c r="I10" s="7">
+        <f t="shared" ca="1" si="6"/>
+        <v>3</v>
+      </c>
+      <c r="J10" s="7">
+        <f t="shared" ca="1" si="7"/>
+        <v>9</v>
+      </c>
+      <c r="K10" s="8">
+        <f t="shared" ca="1" si="8"/>
+        <v>1</v>
+      </c>
+      <c r="L10" s="8">
+        <f t="shared" ca="1" si="9"/>
+        <v>1</v>
+      </c>
+      <c r="M10" s="9">
+        <f t="shared" ref="M9:M12" ca="1" si="10">SUM(F10,D10,H10,J10,L10)</f>
+        <v>48</v>
+      </c>
+    </row>
+    <row r="11" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B11" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="C11" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="D11" s="4">
+        <f t="shared" ca="1" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="E11" s="5">
+        <f t="shared" ca="1" si="2"/>
+        <v>2</v>
+      </c>
+      <c r="F11" s="5">
+        <f t="shared" ca="1" si="3"/>
+        <v>10</v>
+      </c>
+      <c r="G11" s="6">
+        <f t="shared" ca="1" si="4"/>
+        <v>4</v>
+      </c>
+      <c r="H11" s="6">
+        <f t="shared" ca="1" si="5"/>
+        <v>16</v>
+      </c>
+      <c r="I11" s="7">
+        <f t="shared" ca="1" si="6"/>
+        <v>2</v>
+      </c>
+      <c r="J11" s="7">
+        <f t="shared" ca="1" si="7"/>
+        <v>6</v>
+      </c>
+      <c r="K11" s="8">
+        <f t="shared" ca="1" si="8"/>
+        <v>3</v>
+      </c>
+      <c r="L11" s="8">
+        <f t="shared" ca="1" si="9"/>
+        <v>3</v>
+      </c>
+      <c r="M11" s="9">
+        <f ca="1">SUM(F11,D11,H11,J11,L11)</f>
+        <v>38</v>
+      </c>
+    </row>
+    <row r="12" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B12" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="C12" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="D12" s="4">
+        <f t="shared" ca="1" si="1"/>
+        <v>9</v>
+      </c>
+      <c r="E12" s="5">
+        <f t="shared" ca="1" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="F12" s="5">
+        <f t="shared" ca="1" si="3"/>
+        <v>5</v>
+      </c>
+      <c r="G12" s="6">
+        <f t="shared" ca="1" si="4"/>
+        <v>5</v>
+      </c>
+      <c r="H12" s="6">
+        <f t="shared" ca="1" si="5"/>
+        <v>20</v>
+      </c>
+      <c r="I12" s="7">
+        <f t="shared" ca="1" si="6"/>
+        <v>5</v>
+      </c>
+      <c r="J12" s="7">
+        <f t="shared" ca="1" si="7"/>
+        <v>15</v>
+      </c>
+      <c r="K12" s="8">
+        <f t="shared" ca="1" si="8"/>
+        <v>2</v>
+      </c>
+      <c r="L12" s="8">
+        <f t="shared" ca="1" si="9"/>
+        <v>2</v>
+      </c>
+      <c r="M12" s="9">
+        <f ca="1">SUM(F12,D12,H12,J12,L12)</f>
+        <v>51</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
+  <conditionalFormatting sqref="M8:M12">
+    <cfRule type="top10" dxfId="0" priority="1" percent="1" rank="10"/>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>